<commit_message>
[Upgrade] Cap nhat thuat toan goi y tu TF-IDF sang Okapi BM25 chuan xep hang
</commit_message>
<xml_diff>
--- a/docs/BANG_PHAN_CONG_MINI_TASKS_IE104.xlsx
+++ b/docs/BANG_PHAN_CONG_MINI_TASKS_IE104.xlsx
@@ -172,7 +172,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -222,11 +222,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B365D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="001B365D"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B365D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001B365D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B365D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="001B365D"/>
+      </right>
+      <top style="medium">
+        <color rgb="001B365D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B365D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -460,6 +504,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1366,12 +1412,12 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Thuật toán TF-IDF &amp; Cosine Similarity thuần</t>
+          <t>Thuật toán Okapi BM25 thuần (Best Matching 25)</t>
         </is>
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>Viết hàm tính ma trận trọng số TF-IDF và độ tương đồng Cosine Similarity bằng Vanilla JS thuần: Trả về Match Score (%) và danh sách từ khóa trùng khớp.</t>
+          <t>Lập trình thuật toán tìm kiếm và xếp hạng Okapi BM25 bằng Vanilla JS thuần: Điều chỉnh tham số k1 = 1.2, b = 0.75, chuẩn hóa độ dài văn bản, trả về Match Score (%) và từ khóa trùng khớp.</t>
         </is>
       </c>
       <c r="E15" s="26" t="inlineStr">
@@ -1396,7 +1442,7 @@
       </c>
       <c r="I15" s="30" t="inlineStr">
         <is>
-          <t>DÙNG MOCK SCOPE CORPUS: TV2 tự tạo mảng gồm 3 đoạn văn bản mô tả scope mẫu để kiểm thử thuật toán vector và đo tốc độ (&lt;100ms) trước.</t>
+          <t>DÙNG MOCK SCOPE CORPUS: TV2 tự tạo mảng gồm 3 đoạn văn bản mô tả scope mẫu để kiểm thử thuật toán Okapi BM25 và đo tốc độ (&lt;100ms) trước.</t>
         </is>
       </c>
       <c r="J15" s="31" t="inlineStr">
@@ -1485,7 +1531,7 @@
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
-          <t>Trình bày chi tiết cơ sở toán học TF-IDF, công thức Cosine Similarity, sơ đồ giải thuật và phân tích hiệu năng trong Báo cáo PDF.</t>
+          <t>Trình bày chi tiết cơ sở toán học Okapi BM25, hàm chấm điểm Relevance Score, sơ đồ giải thuật và phân tích hiệu năng trong Báo cáo PDF.</t>
         </is>
       </c>
       <c r="E17" s="26" t="inlineStr">
@@ -2385,11 +2431,11 @@
           <t>TỔNG CỘNG TIẾN ĐỘ &amp; TRỌNG SỐ 25 MINI-TASKS (5 THÀNH VIÊN X 20% = 100%)</t>
         </is>
       </c>
-      <c r="B33" s="69" t="n"/>
-      <c r="C33" s="69" t="n"/>
-      <c r="D33" s="69" t="n"/>
-      <c r="E33" s="69" t="n"/>
-      <c r="F33" s="69" t="n"/>
+      <c r="B33" s="81" t="n"/>
+      <c r="C33" s="81" t="n"/>
+      <c r="D33" s="81" t="n"/>
+      <c r="E33" s="81" t="n"/>
+      <c r="F33" s="82" t="n"/>
       <c r="G33" s="70" t="inlineStr">
         <is>
           <t>100%</t>

</xml_diff>